<commit_message>
#3 Library in Progress
</commit_message>
<xml_diff>
--- a/BOM_CB_BIU_S2v2.0_Changes.xlsx
+++ b/BOM_CB_BIU_S2v2.0_Changes.xlsx
@@ -1724,7 +1724,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1845,6 +1845,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4721,7 +4724,7 @@
       <c r="F43" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="G43" s="5" t="s">
+      <c r="G43" s="43" t="s">
         <v>175</v>
       </c>
       <c r="H43" s="5">
@@ -4779,7 +4782,7 @@
       <c r="F44" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="G44" s="5" t="s">
+      <c r="G44" s="43" t="s">
         <v>177</v>
       </c>
       <c r="H44" s="5" t="s">
@@ -4837,7 +4840,7 @@
       <c r="F45" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="G45" s="5" t="s">
+      <c r="G45" s="43" t="s">
         <v>183</v>
       </c>
       <c r="H45" s="5" t="s">
@@ -4898,7 +4901,7 @@
       <c r="F46" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="G46" s="5">
+      <c r="G46" s="43">
         <v>484060003</v>
       </c>
       <c r="H46" s="5" t="s">
@@ -5014,7 +5017,7 @@
       <c r="F48" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="G48" s="5" t="s">
+      <c r="G48" s="43" t="s">
         <v>196</v>
       </c>
       <c r="H48" s="5" t="s">
@@ -5130,7 +5133,7 @@
       <c r="F50" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="G50" s="7" t="s">
+      <c r="G50" s="44" t="s">
         <v>204</v>
       </c>
       <c r="H50" s="5" t="s">
@@ -5188,7 +5191,7 @@
       <c r="F51" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="G51" s="7" t="s">
+      <c r="G51" s="44" t="s">
         <v>207</v>
       </c>
       <c r="H51" s="5" t="s">
@@ -5246,7 +5249,7 @@
       <c r="F52" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="G52" s="5" t="s">
+      <c r="G52" s="43" t="s">
         <v>215</v>
       </c>
       <c r="H52" s="5" t="s">
@@ -5304,7 +5307,7 @@
       <c r="F53" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="G53" s="5" t="s">
+      <c r="G53" s="43" t="s">
         <v>220</v>
       </c>
       <c r="H53" s="5" t="s">

</xml_diff>

<commit_message>
#3 Carrier Board Library Completed.
</commit_message>
<xml_diff>
--- a/BOM_CB_BIU_S2v2.0_Changes.xlsx
+++ b/BOM_CB_BIU_S2v2.0_Changes.xlsx
@@ -1588,7 +1588,7 @@
     <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* \-??_ ;_-@_ "/>
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1643,6 +1643,13 @@
     <font>
       <sz val="11"/>
       <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -1737,7 +1744,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1867,6 +1874,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -8328,7 +8338,7 @@
       <c r="F105" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="G105" s="5" t="s">
+      <c r="G105" s="43" t="s">
         <v>440</v>
       </c>
       <c r="H105" s="5" t="s">
@@ -8386,7 +8396,7 @@
       <c r="F106" s="5" t="s">
         <v>445</v>
       </c>
-      <c r="G106" s="5" t="s">
+      <c r="G106" s="43" t="s">
         <v>446</v>
       </c>
       <c r="H106" s="5" t="s">
@@ -8444,7 +8454,7 @@
       <c r="F107" s="5" t="s">
         <v>445</v>
       </c>
-      <c r="G107" s="5" t="s">
+      <c r="G107" s="43" t="s">
         <v>449</v>
       </c>
       <c r="H107" s="5" t="s">
@@ -8502,7 +8512,7 @@
       <c r="F108" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="G108" s="5" t="s">
+      <c r="G108" s="43" t="s">
         <v>453</v>
       </c>
       <c r="H108" s="5" t="s">
@@ -8560,7 +8570,7 @@
       <c r="F109" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="G109" s="5" t="s">
+      <c r="G109" s="43" t="s">
         <v>457</v>
       </c>
       <c r="H109" s="5" t="s">
@@ -8618,7 +8628,7 @@
       <c r="F110" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="G110" s="5" t="s">
+      <c r="G110" s="43" t="s">
         <v>461</v>
       </c>
       <c r="H110" s="5" t="s">
@@ -8676,7 +8686,7 @@
       <c r="F111" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="G111" s="5" t="s">
+      <c r="G111" s="43" t="s">
         <v>466</v>
       </c>
       <c r="H111" s="5" t="s">
@@ -8734,7 +8744,7 @@
       <c r="F112" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="G112" s="5" t="s">
+      <c r="G112" s="43" t="s">
         <v>468</v>
       </c>
       <c r="H112" s="5" t="s">
@@ -8792,7 +8802,7 @@
       <c r="F113" s="5" t="s">
         <v>473</v>
       </c>
-      <c r="G113" s="5" t="s">
+      <c r="G113" s="43" t="s">
         <v>471</v>
       </c>
       <c r="H113" s="5" t="s">
@@ -8850,7 +8860,7 @@
       <c r="F114" s="5" t="s">
         <v>478</v>
       </c>
-      <c r="G114" s="5" t="s">
+      <c r="G114" s="47" t="s">
         <v>479</v>
       </c>
       <c r="H114" s="5" t="s">

</xml_diff>